<commit_message>
updated wrong config files
</commit_message>
<xml_diff>
--- a/configs/wpc/5/train.xlsx
+++ b/configs/wpc/5/train.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1785" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1674" uniqueCount="622">
   <si>
     <t>Content</t>
   </si>
@@ -10219,17 +10219,17 @@
       </c>
     </row>
     <row r="372" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A372" t="s">
-        <v>354</v>
-      </c>
-      <c r="B372" s="2" t="s">
-        <v>355</v>
+      <c r="A372" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B372" s="2" t="str">
+        <v>cauliflower_gQP_1_tQP_1.ply</v>
       </c>
       <c r="C372">
-        <v>77.914700954506003</v>
-      </c>
-      <c r="D372" t="s">
-        <v>10</v>
+        <v>87.6248392427318</v>
+      </c>
+      <c r="D372" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E372">
         <v>1</v>
@@ -10239,17 +10239,17 @@
       </c>
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A373" t="s">
-        <v>354</v>
-      </c>
-      <c r="B373" s="2" t="s">
-        <v>356</v>
+      <c r="A373" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B373" s="2" t="str">
+        <v>cauliflower_gQP_1_tQP_2.ply</v>
       </c>
       <c r="C373">
-        <v>75.444459102442195</v>
-      </c>
-      <c r="D373" t="s">
-        <v>10</v>
+        <v>69.9340182104258</v>
+      </c>
+      <c r="D373" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E373">
         <v>1</v>
@@ -10259,17 +10259,17 @@
       </c>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A374" t="s">
-        <v>354</v>
-      </c>
-      <c r="B374" s="2" t="s">
-        <v>357</v>
+      <c r="A374" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B374" s="2" t="str">
+        <v>cauliflower_gQP_1_tQP_3.ply</v>
       </c>
       <c r="C374">
-        <v>51.298874521677398</v>
-      </c>
-      <c r="D374" t="s">
-        <v>10</v>
+        <v>55.8664800791356</v>
+      </c>
+      <c r="D374" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E374">
         <v>1</v>
@@ -10279,17 +10279,17 @@
       </c>
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A375" t="s">
-        <v>354</v>
-      </c>
-      <c r="B375" s="2" t="s">
-        <v>358</v>
+      <c r="A375" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B375" s="2" t="str">
+        <v>cauliflower_gQP_2_tQP_1.ply</v>
       </c>
       <c r="C375">
-        <v>62.505454143241103</v>
-      </c>
-      <c r="D375" t="s">
-        <v>10</v>
+        <v>77.6400648006452</v>
+      </c>
+      <c r="D375" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E375">
         <v>2</v>
@@ -10299,17 +10299,17 @@
       </c>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A376" t="s">
-        <v>354</v>
-      </c>
-      <c r="B376" s="2" t="s">
-        <v>359</v>
+      <c r="A376" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B376" s="2" t="str">
+        <v>cauliflower_gQP_2_tQP_2.ply</v>
       </c>
       <c r="C376">
-        <v>63.425654765989798</v>
-      </c>
-      <c r="D376" t="s">
-        <v>10</v>
+        <v>61.7264692699532</v>
+      </c>
+      <c r="D376" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E376">
         <v>2</v>
@@ -10319,17 +10319,17 @@
       </c>
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A377" t="s">
-        <v>354</v>
-      </c>
-      <c r="B377" s="2" t="s">
-        <v>360</v>
+      <c r="A377" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B377" s="2" t="str">
+        <v>cauliflower_gQP_2_tQP_3.ply</v>
       </c>
       <c r="C377">
-        <v>48.993284607112898</v>
-      </c>
-      <c r="D377" t="s">
-        <v>10</v>
+        <v>50.2228411565292</v>
+      </c>
+      <c r="D377" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E377">
         <v>2</v>
@@ -10339,17 +10339,17 @@
       </c>
     </row>
     <row r="378" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A378" t="s">
-        <v>354</v>
-      </c>
-      <c r="B378" s="2" t="s">
-        <v>361</v>
+      <c r="A378" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B378" s="2" t="str">
+        <v>cauliflower_gQP_3_tQP_1.ply</v>
       </c>
       <c r="C378">
-        <v>49.253303178785302</v>
-      </c>
-      <c r="D378" t="s">
-        <v>10</v>
+        <v>34.4736481448513</v>
+      </c>
+      <c r="D378" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E378">
         <v>3</v>
@@ -10359,17 +10359,17 @@
       </c>
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A379" t="s">
-        <v>354</v>
-      </c>
-      <c r="B379" s="2" t="s">
-        <v>362</v>
+      <c r="A379" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B379" s="2" t="str">
+        <v>cauliflower_gQP_3_tQP_2.ply</v>
       </c>
       <c r="C379">
-        <v>42.084168780933098</v>
-      </c>
-      <c r="D379" t="s">
-        <v>10</v>
+        <v>27.4116195543465</v>
+      </c>
+      <c r="D379" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E379">
         <v>3</v>
@@ -10379,17 +10379,17 @@
       </c>
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A380" t="s">
-        <v>354</v>
-      </c>
-      <c r="B380" s="2" t="s">
-        <v>363</v>
+      <c r="A380" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B380" s="2" t="str">
+        <v>cauliflower_gQP_3_tQP_3.ply</v>
       </c>
       <c r="C380">
-        <v>37.310713536647903</v>
-      </c>
-      <c r="D380" t="s">
-        <v>10</v>
+        <v>30.2313975655941</v>
+      </c>
+      <c r="D380" t="str">
+        <v>V-PCC</v>
       </c>
       <c r="E380">
         <v>3</v>
@@ -10399,17 +10399,17 @@
       </c>
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A381" t="s">
-        <v>354</v>
-      </c>
-      <c r="B381" s="2" t="s">
-        <v>364</v>
+      <c r="A381" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B381" s="2" t="str">
+        <v>cauliflower_gsigma_0_tsigma_16.ply</v>
       </c>
       <c r="C381">
-        <v>48.6325940292948</v>
-      </c>
-      <c r="D381" t="s">
-        <v>20</v>
+        <v>57.425103805969</v>
+      </c>
+      <c r="D381" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E381">
         <v>0</v>
@@ -10419,17 +10419,17 @@
       </c>
     </row>
     <row r="382" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A382" t="s">
-        <v>354</v>
-      </c>
-      <c r="B382" s="2" t="s">
-        <v>365</v>
+      <c r="A382" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B382" s="2" t="str">
+        <v>cauliflower_gsigma_0_tsigma_32.ply</v>
       </c>
       <c r="C382">
-        <v>34.740857695205797</v>
-      </c>
-      <c r="D382" t="s">
-        <v>20</v>
+        <v>40.190717226665</v>
+      </c>
+      <c r="D382" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E382">
         <v>0</v>
@@ -10439,17 +10439,17 @@
       </c>
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A383" t="s">
-        <v>354</v>
-      </c>
-      <c r="B383" s="2" t="s">
-        <v>366</v>
+      <c r="A383" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B383" s="2" t="str">
+        <v>cauliflower_gsigma_0_tsigma_8.ply</v>
       </c>
       <c r="C383">
-        <v>79.476693349159802</v>
-      </c>
-      <c r="D383" t="s">
-        <v>20</v>
+        <v>77.7622683284028</v>
+      </c>
+      <c r="D383" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E383">
         <v>0</v>
@@ -10459,17 +10459,17 @@
       </c>
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A384" t="s">
-        <v>354</v>
-      </c>
-      <c r="B384" s="2" t="s">
-        <v>367</v>
+      <c r="A384" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B384" s="2" t="str">
+        <v>cauliflower_gsigma_2_tsigma_16.ply</v>
       </c>
       <c r="C384">
-        <v>32.552309796614402</v>
-      </c>
-      <c r="D384" t="s">
-        <v>20</v>
+        <v>53.1317191703664</v>
+      </c>
+      <c r="D384" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E384">
         <v>2</v>
@@ -10479,17 +10479,17 @@
       </c>
     </row>
     <row r="385" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A385" t="s">
-        <v>354</v>
-      </c>
-      <c r="B385" s="2" t="s">
-        <v>368</v>
+      <c r="A385" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B385" s="2" t="str">
+        <v>cauliflower_gsigma_2_tsigma_32.ply</v>
       </c>
       <c r="C385">
-        <v>27.413599096493499</v>
-      </c>
-      <c r="D385" t="s">
-        <v>20</v>
+        <v>31.3681861609079</v>
+      </c>
+      <c r="D385" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E385">
         <v>2</v>
@@ -10499,17 +10499,17 @@
       </c>
     </row>
     <row r="386" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A386" t="s">
-        <v>354</v>
-      </c>
-      <c r="B386" s="2" t="s">
-        <v>369</v>
+      <c r="A386" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B386" s="2" t="str">
+        <v>cauliflower_gsigma_2_tsigma_8.ply</v>
       </c>
       <c r="C386">
-        <v>43.470265563476403</v>
-      </c>
-      <c r="D386" t="s">
-        <v>20</v>
+        <v>64.1622967039307</v>
+      </c>
+      <c r="D386" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E386">
         <v>2</v>
@@ -10519,17 +10519,17 @@
       </c>
     </row>
     <row r="387" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A387" t="s">
-        <v>354</v>
-      </c>
-      <c r="B387" s="2" t="s">
-        <v>370</v>
+      <c r="A387" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B387" s="2" t="str">
+        <v>cauliflower_gsigma_4_tsigma_16.ply</v>
       </c>
       <c r="C387">
-        <v>22.986949508254099</v>
-      </c>
-      <c r="D387" t="s">
-        <v>20</v>
+        <v>44.4047016090656</v>
+      </c>
+      <c r="D387" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E387">
         <v>4</v>
@@ -10539,17 +10539,17 @@
       </c>
     </row>
     <row r="388" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A388" t="s">
-        <v>354</v>
-      </c>
-      <c r="B388" s="2" t="s">
-        <v>371</v>
+      <c r="A388" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B388" s="2" t="str">
+        <v>cauliflower_gsigma_4_tsigma_32.ply</v>
       </c>
       <c r="C388">
-        <v>17.408186796220001</v>
-      </c>
-      <c r="D388" t="s">
-        <v>20</v>
+        <v>27.3258415882843</v>
+      </c>
+      <c r="D388" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E388">
         <v>4</v>
@@ -10559,17 +10559,17 @@
       </c>
     </row>
     <row r="389" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A389" t="s">
-        <v>354</v>
-      </c>
-      <c r="B389" s="2" t="s">
-        <v>372</v>
+      <c r="A389" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B389" s="2" t="str">
+        <v>cauliflower_gsigma_4_tsigma_8.ply</v>
       </c>
       <c r="C389">
-        <v>24.0019876904387</v>
-      </c>
-      <c r="D389" t="s">
-        <v>20</v>
+        <v>47.8571729909968</v>
+      </c>
+      <c r="D389" t="str">
+        <v>Gaussian noise</v>
       </c>
       <c r="E389">
         <v>4</v>
@@ -10579,17 +10579,17 @@
       </c>
     </row>
     <row r="390" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A390" t="s">
-        <v>354</v>
-      </c>
-      <c r="B390" s="2" t="s">
-        <v>373</v>
+      <c r="A390" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B390" s="2" t="str">
+        <v>cauliflower_level_7.ply</v>
       </c>
       <c r="C390">
-        <v>3.15346252854002</v>
-      </c>
-      <c r="D390" t="s">
-        <v>30</v>
+        <v>8.79345962299418</v>
+      </c>
+      <c r="D390" t="str">
+        <v>Downsampling</v>
       </c>
       <c r="E390">
         <v>7</v>
@@ -10599,17 +10599,17 @@
       </c>
     </row>
     <row r="391" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A391" t="s">
-        <v>354</v>
-      </c>
-      <c r="B391" s="2" t="s">
-        <v>374</v>
+      <c r="A391" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B391" s="2" t="str">
+        <v>cauliflower_level_8.ply</v>
       </c>
       <c r="C391">
-        <v>16.260334926567499</v>
-      </c>
-      <c r="D391" t="s">
-        <v>30</v>
+        <v>16.0306030369897</v>
+      </c>
+      <c r="D391" t="str">
+        <v>Downsampling</v>
       </c>
       <c r="E391">
         <v>8</v>
@@ -10619,17 +10619,17 @@
       </c>
     </row>
     <row r="392" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A392" t="s">
-        <v>354</v>
-      </c>
-      <c r="B392" s="2" t="s">
-        <v>375</v>
+      <c r="A392" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B392" s="2" t="str">
+        <v>cauliflower_level_9.ply</v>
       </c>
       <c r="C392">
-        <v>77.843266410166805</v>
-      </c>
-      <c r="D392" t="s">
-        <v>30</v>
+        <v>74.6811494247904</v>
+      </c>
+      <c r="D392" t="str">
+        <v>Downsampling</v>
       </c>
       <c r="E392">
         <v>9</v>
@@ -10639,17 +10639,17 @@
       </c>
     </row>
     <row r="393" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A393" t="s">
-        <v>354</v>
-      </c>
-      <c r="B393" s="2" t="s">
-        <v>568</v>
+      <c r="A393" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B393" s="2" t="str">
+        <v>cauliflower_pqs_1_qs_16_rounded.ply</v>
       </c>
       <c r="C393">
-        <v>88.779224881732404</v>
-      </c>
-      <c r="D393" t="s">
-        <v>33</v>
+        <v>90.0384616380816</v>
+      </c>
+      <c r="D393" t="str">
+        <v>G-PCC (O)/L-PCC</v>
       </c>
       <c r="E393">
         <v>1</v>
@@ -10659,17 +10659,17 @@
       </c>
     </row>
     <row r="394" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A394" t="s">
-        <v>354</v>
-      </c>
-      <c r="B394" s="2" t="s">
-        <v>584</v>
+      <c r="A394" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B394" s="2" t="str">
+        <v>cauliflower_pqs_1_qs_32_rounded.ply</v>
       </c>
       <c r="C394">
-        <v>57.830740344231401</v>
-      </c>
-      <c r="D394" t="s">
-        <v>33</v>
+        <v>63.72945613739</v>
+      </c>
+      <c r="D394" t="str">
+        <v>G-PCC (O)/L-PCC</v>
       </c>
       <c r="E394">
         <v>1</v>
@@ -10679,17 +10679,17 @@
       </c>
     </row>
     <row r="395" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A395" t="s">
-        <v>354</v>
-      </c>
-      <c r="B395" s="2" t="s">
-        <v>600</v>
+      <c r="A395" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B395" s="2" t="str">
+        <v>cauliflower_pqs_1_qs_48_rounded.ply</v>
       </c>
       <c r="C395">
-        <v>53.831014428938701</v>
-      </c>
-      <c r="D395" t="s">
-        <v>33</v>
+        <v>27.0784601811131</v>
+      </c>
+      <c r="D395" t="str">
+        <v>G-PCC (O)/L-PCC</v>
       </c>
       <c r="E395">
         <v>1</v>
@@ -10699,17 +10699,17 @@
       </c>
     </row>
     <row r="396" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A396" t="s">
-        <v>354</v>
-      </c>
-      <c r="B396" s="2" t="s">
-        <v>616</v>
+      <c r="A396" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B396" s="2" t="str">
+        <v>cauliflower_pqs_1_qs_64_rounded.ply</v>
       </c>
       <c r="C396">
-        <v>48.013544967176898</v>
-      </c>
-      <c r="D396" t="s">
-        <v>33</v>
+        <v>14.4033486133223</v>
+      </c>
+      <c r="D396" t="str">
+        <v>G-PCC (O)/L-PCC</v>
       </c>
       <c r="E396">
         <v>1</v>
@@ -10718,24 +10718,24 @@
         <v>64</v>
       </c>
       <c r="H396">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I396">
         <v>35</v>
       </c>
     </row>
     <row r="397" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A397" t="s">
-        <v>354</v>
-      </c>
-      <c r="B397" s="2" t="s">
-        <v>376</v>
+      <c r="A397" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B397" s="2" t="str">
+        <v>cauliflower_tsl_4_tqs_128.ply</v>
       </c>
       <c r="C397">
-        <v>26.819913530637798</v>
-      </c>
-      <c r="D397" t="s">
-        <v>35</v>
+        <v>42.188692944374</v>
+      </c>
+      <c r="D397" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E397">
         <v>4</v>
@@ -10744,24 +10744,24 @@
         <v>128</v>
       </c>
       <c r="H397">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I397">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="398" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A398" t="s">
-        <v>354</v>
-      </c>
-      <c r="B398" s="2" t="s">
-        <v>377</v>
+      <c r="A398" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B398" s="2" t="str">
+        <v>cauliflower_tsl_4_tqs_256.ply</v>
       </c>
       <c r="C398">
-        <v>12.1998153379797</v>
-      </c>
-      <c r="D398" t="s">
-        <v>35</v>
+        <v>33.1300686929086</v>
+      </c>
+      <c r="D398" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E398">
         <v>4</v>
@@ -10770,24 +10770,24 @@
         <v>256</v>
       </c>
       <c r="H398">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="I398">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="399" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A399" t="s">
-        <v>354</v>
-      </c>
-      <c r="B399" s="2" t="s">
-        <v>378</v>
+      <c r="A399" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B399" s="2" t="str">
+        <v>cauliflower_tsl_4_tqs_512.ply</v>
       </c>
       <c r="C399">
-        <v>5.84222472057741</v>
-      </c>
-      <c r="D399" t="s">
-        <v>35</v>
+        <v>26.6104175998077</v>
+      </c>
+      <c r="D399" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E399">
         <v>4</v>
@@ -10796,24 +10796,24 @@
         <v>512</v>
       </c>
       <c r="H399">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I399">
         <v>35</v>
       </c>
     </row>
     <row r="400" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A400" t="s">
-        <v>354</v>
-      </c>
-      <c r="B400" s="2" t="s">
-        <v>379</v>
+      <c r="A400" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B400" s="2" t="str">
+        <v>cauliflower_tsl_4_tqs_64.ply</v>
       </c>
       <c r="C400">
-        <v>22.6305666322368</v>
-      </c>
-      <c r="D400" t="s">
-        <v>35</v>
+        <v>61.9039972872389</v>
+      </c>
+      <c r="D400" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E400">
         <v>4</v>
@@ -10822,24 +10822,24 @@
         <v>64</v>
       </c>
       <c r="H400">
+        <v>40</v>
+      </c>
+      <c r="I400">
         <v>45</v>
       </c>
-      <c r="I400">
-        <v>40</v>
-      </c>
     </row>
     <row r="401" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A401" t="s">
-        <v>354</v>
-      </c>
-      <c r="B401" s="2" t="s">
-        <v>380</v>
+      <c r="A401" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B401" s="2" t="str">
+        <v>cauliflower_tsl_6_tqs_128.ply</v>
       </c>
       <c r="C401">
-        <v>62.986212148395801</v>
-      </c>
-      <c r="D401" t="s">
-        <v>35</v>
+        <v>64.2706535471644</v>
+      </c>
+      <c r="D401" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E401">
         <v>6</v>
@@ -10848,24 +10848,24 @@
         <v>128</v>
       </c>
       <c r="H401">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I401">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="402" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A402" t="s">
-        <v>354</v>
-      </c>
-      <c r="B402" s="2" t="s">
-        <v>381</v>
+      <c r="A402" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B402" s="2" t="str">
+        <v>cauliflower_tsl_6_tqs_256.ply</v>
       </c>
       <c r="C402">
-        <v>28.555861781951201</v>
-      </c>
-      <c r="D402" t="s">
-        <v>35</v>
+        <v>41.8663397248415</v>
+      </c>
+      <c r="D402" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E402">
         <v>6</v>
@@ -10881,17 +10881,17 @@
       </c>
     </row>
     <row r="403" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A403" t="s">
-        <v>354</v>
-      </c>
-      <c r="B403" s="2" t="s">
-        <v>382</v>
+      <c r="A403" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B403" s="2" t="str">
+        <v>cauliflower_tsl_6_tqs_512.ply</v>
       </c>
       <c r="C403">
-        <v>16.599548474370099</v>
-      </c>
-      <c r="D403" t="s">
-        <v>35</v>
+        <v>29.7421656574121</v>
+      </c>
+      <c r="D403" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E403">
         <v>6</v>
@@ -10903,21 +10903,21 @@
         <v>50</v>
       </c>
       <c r="I403">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="404" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A404" t="s">
-        <v>354</v>
-      </c>
-      <c r="B404" s="2" t="s">
-        <v>383</v>
+      <c r="A404" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B404" s="2" t="str">
+        <v>cauliflower_tsl_6_tqs_64.ply</v>
       </c>
       <c r="C404">
-        <v>86.880448765472707</v>
-      </c>
-      <c r="D404" t="s">
-        <v>35</v>
+        <v>75.5339573340953</v>
+      </c>
+      <c r="D404" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E404">
         <v>6</v>
@@ -10929,21 +10929,21 @@
         <v>50</v>
       </c>
       <c r="I404">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="405" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A405" t="s">
-        <v>354</v>
-      </c>
-      <c r="B405" s="2" t="s">
-        <v>384</v>
+      <c r="A405" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B405" s="2" t="str">
+        <v>cauliflower_tsl_8_tqs_128.ply</v>
       </c>
       <c r="C405">
-        <v>61.7974566844332</v>
-      </c>
-      <c r="D405" t="s">
-        <v>35</v>
+        <v>79.7652667648818</v>
+      </c>
+      <c r="D405" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E405">
         <v>8</v>
@@ -10953,17 +10953,17 @@
       </c>
     </row>
     <row r="406" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A406" t="s">
-        <v>354</v>
-      </c>
-      <c r="B406" s="2" t="s">
-        <v>385</v>
+      <c r="A406" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B406" s="2" t="str">
+        <v>cauliflower_tsl_8_tqs_256.ply</v>
       </c>
       <c r="C406">
-        <v>36.113641068392397</v>
-      </c>
-      <c r="D406" t="s">
-        <v>35</v>
+        <v>43.9879089599129</v>
+      </c>
+      <c r="D406" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E406">
         <v>8</v>
@@ -10973,17 +10973,17 @@
       </c>
     </row>
     <row r="407" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A407" t="s">
-        <v>354</v>
-      </c>
-      <c r="B407" s="2" t="s">
-        <v>386</v>
+      <c r="A407" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B407" s="2" t="str">
+        <v>cauliflower_tsl_8_tqs_512.ply</v>
       </c>
       <c r="C407">
-        <v>21.545909315501099</v>
-      </c>
-      <c r="D407" t="s">
-        <v>35</v>
+        <v>27.7443960854802</v>
+      </c>
+      <c r="D407" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E407">
         <v>8</v>
@@ -10993,17 +10993,17 @@
       </c>
     </row>
     <row r="408" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A408" t="s">
-        <v>354</v>
-      </c>
-      <c r="B408" s="2" t="s">
-        <v>387</v>
+      <c r="A408" t="str">
+        <v>cauliflower</v>
+      </c>
+      <c r="B408" s="2" t="str">
+        <v>cauliflower_tsl_8_tqs_64.ply</v>
       </c>
       <c r="C408">
-        <v>79.845330517493196</v>
-      </c>
-      <c r="D408" t="s">
-        <v>35</v>
+        <v>92.8513690778754</v>
+      </c>
+      <c r="D408" t="str">
+        <v>G-PCC (T)/S-PCC</v>
       </c>
       <c r="E408">
         <v>8</v>

</xml_diff>